<commit_message>
Add French versions of P1 and P2
- i18n layer translates cell text, formula string literals, sheet names and
  conditional-format formulas at build time; calculations are shared
- TEXT() calls rewritten to FIXED() so generated sentences use the user's locale separators
- French dictionary, user guides and Etsy/Gumroad listings; listing checker handles both files

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BXecWCCHxS2NDKTkshp3of
</commit_message>
<xml_diff>
--- a/product/01-entry-calculator/MiniGrid_Feasibility_Calculator_v1.xlsx
+++ b/product/01-entry-calculator/MiniGrid_Feasibility_Calculator_v1.xlsx
@@ -2145,8 +2145,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="38041402"/>
-        <c:axId val="78697009"/>
+        <c:axId val="4474254"/>
+        <c:axId val="94918355"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2351,11 +2351,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="38041402"/>
-        <c:axId val="78697009"/>
+        <c:axId val="4474254"/>
+        <c:axId val="94918355"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="38041402"/>
+        <c:axId val="4474254"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2387,7 +2387,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78697009"/>
+        <c:crossAx val="94918355"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2395,7 +2395,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78697009"/>
+        <c:axId val="94918355"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2471,7 +2471,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38041402"/>
+        <c:crossAx val="4474254"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2942,11 +2942,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="35144353"/>
-        <c:axId val="87863784"/>
+        <c:axId val="22569887"/>
+        <c:axId val="14356195"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="35144353"/>
+        <c:axId val="22569887"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2978,7 +2978,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87863784"/>
+        <c:crossAx val="14356195"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2986,7 +2986,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87863784"/>
+        <c:axId val="14356195"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3028,7 +3028,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35144353"/>
+        <c:crossAx val="22569887"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4518,7 +4518,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="7" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="12" style="0" width="12"/>
   </cols>
@@ -4531,7 +4531,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="35" t="str">
-        <f aca="false">Site&amp;"  |  "&amp;TotalCustomers&amp;" customers  |  "&amp;TEXT(PV_kWp,"#,##0")&amp;" kWp PV / "&amp;TEXT(BESS_kWh,"#,##0")&amp;" kWh battery / "&amp;TEXT(Diesel_kW,"#,##0")&amp;" kW diesel  |  amounts in "&amp;Currency</f>
+        <f aca="false">Site&amp;"  |  "&amp;TotalCustomers&amp;" customers  |  "&amp;FIXED(PV_kWp,0)&amp;" kWp PV / "&amp;FIXED(BESS_kWh,0)&amp;" kWh battery / "&amp;FIXED(Diesel_kW,0)&amp;" kW diesel  |  amounts in "&amp;Currency</f>
         <v>Example site  |  970 customers  |  349 kWp PV / 780 kWh battery / 145 kW diesel  |  amounts in USD</v>
       </c>
       <c r="F2" s="35" t="str">
@@ -5436,10 +5436,10 @@
   </sheetData>
   <conditionalFormatting sqref="F18:F22">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>LEFT(F18,3)="YES"</formula>
+      <formula>LEFT(F18,LEN("YES"))="YES"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>LEFT(F18,2)="NO"</formula>
+      <formula>OR(LEFT(F18,LEN("NO - "))="NO - ",F18="NO")</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>